<commit_message>
correct typos in the ibd code
</commit_message>
<xml_diff>
--- a/results/outputs/ibd/ibd_enrichment.xlsx
+++ b/results/outputs/ibd/ibd_enrichment.xlsx
@@ -464,10 +464,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.01178989910767969</v>
+        <v>0.01177420696520263</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1061090919691172</v>
+        <v>0.1059678626868236</v>
       </c>
     </row>
     <row r="3">
@@ -482,10 +482,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.0153008631781769</v>
+        <v>0.01528053267818888</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1224069054254152</v>
+        <v>0.1222442614255111</v>
       </c>
     </row>
     <row r="4">
@@ -500,10 +500,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.01646853074607243</v>
+        <v>0.01644666117929082</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1224069054254152</v>
+        <v>0.1222442614255111</v>
       </c>
     </row>
     <row r="5">
@@ -518,10 +518,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.01646853074607243</v>
+        <v>0.01644666117929082</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1224069054254152</v>
+        <v>0.1222442614255111</v>
       </c>
     </row>
     <row r="6">
@@ -536,10 +536,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.02228702974004062</v>
+        <v>0.02225751747440972</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1224069054254152</v>
+        <v>0.1222442614255111</v>
       </c>
     </row>
     <row r="7">
@@ -554,10 +554,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.02691810812776645</v>
+        <v>0.02688254452312406</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1224069054254152</v>
+        <v>0.1222442614255111</v>
       </c>
     </row>
     <row r="8">
@@ -572,10 +572,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.04409848221966672</v>
+        <v>0.04404071697551871</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1322954466590002</v>
+        <v>0.1321221509265561</v>
       </c>
     </row>
     <row r="9">
@@ -590,10 +590,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.0486306809989439</v>
+        <v>0.04856712458848836</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1322954466590002</v>
+        <v>0.1321221509265561</v>
       </c>
     </row>
     <row r="10">
@@ -608,10 +608,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.9825800280351759</v>
+        <v>0.9824764702199092</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9825800280351759</v>
+        <v>0.9824764702199092</v>
       </c>
     </row>
   </sheetData>
@@ -662,10 +662,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5.152248956669586e-05</v>
+        <v>5.145356315924878e-05</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00149415219743418</v>
+        <v>0.001492153331618215</v>
       </c>
     </row>
     <row r="3">
@@ -680,10 +680,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.0005152248956669587</v>
+        <v>0.0005145356315924877</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01442629707867484</v>
+        <v>0.01440699768458966</v>
       </c>
     </row>
     <row r="4">
@@ -698,10 +698,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0005667473852336546</v>
+        <v>0.0005659891947517366</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01530217940130867</v>
+        <v>0.01528170825829689</v>
       </c>
     </row>
     <row r="5">
@@ -716,10 +716,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.0006182698748003504</v>
+        <v>0.0006174427579109853</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01607501674480911</v>
+        <v>0.01605351170568562</v>
       </c>
     </row>
     <row r="6">
@@ -734,10 +734,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.0006697923643670462</v>
+        <v>0.0006688963210702341</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01674480910917615</v>
+        <v>0.01672240802675585</v>
       </c>
     </row>
     <row r="7">
@@ -752,10 +752,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.0006697923643670462</v>
+        <v>0.0006688963210702341</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01674480910917615</v>
+        <v>0.01672240802675585</v>
       </c>
     </row>
     <row r="8">
@@ -770,10 +770,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.0007213148539337422</v>
+        <v>0.0007203498842294829</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01674480910917615</v>
+        <v>0.01672240802675585</v>
       </c>
     </row>
     <row r="9">
@@ -788,10 +788,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.0009274048122005254</v>
+        <v>0.0009261641368664779</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02040290586841156</v>
+        <v>0.02037561101106251</v>
       </c>
     </row>
     <row r="10">
@@ -806,10 +806,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.0009789273017672215</v>
+        <v>0.0009776177000257267</v>
       </c>
       <c r="D10" t="n">
-        <v>0.02055747333711165</v>
+        <v>0.02052997170054026</v>
       </c>
     </row>
     <row r="11">
@@ -824,10 +824,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.001030449791333917</v>
+        <v>0.001029071263184975</v>
       </c>
       <c r="D11" t="n">
-        <v>0.02060899582667835</v>
+        <v>0.02058142526369951</v>
       </c>
     </row>
     <row r="12">
@@ -842,10 +842,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.001081972280900613</v>
+        <v>0.001080524826344225</v>
       </c>
       <c r="D12" t="n">
-        <v>0.02060899582667835</v>
+        <v>0.02058142526369951</v>
       </c>
     </row>
     <row r="13">
@@ -860,10 +860,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.001133494770467309</v>
+        <v>0.001131978389503473</v>
       </c>
       <c r="D13" t="n">
-        <v>0.02060899582667835</v>
+        <v>0.02058142526369951</v>
       </c>
     </row>
     <row r="14">
@@ -878,10 +878,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.001236539749600701</v>
+        <v>0.001234885515821971</v>
       </c>
       <c r="D14" t="n">
-        <v>0.02102117574321191</v>
+        <v>0.0209930537689735</v>
       </c>
     </row>
     <row r="15">
@@ -896,10 +896,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.001288062239167397</v>
+        <v>0.001286339078981219</v>
       </c>
       <c r="D15" t="n">
-        <v>0.02102117574321191</v>
+        <v>0.0209930537689735</v>
       </c>
     </row>
     <row r="16">
@@ -914,10 +914,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.00149415219743418</v>
+        <v>0.001492153331618215</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0224122829615127</v>
+        <v>0.02238229997427322</v>
       </c>
     </row>
     <row r="17">
@@ -932,10 +932,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.001597197176567572</v>
+        <v>0.001595060457936712</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0224122829615127</v>
+        <v>0.02238229997427322</v>
       </c>
     </row>
     <row r="18">
@@ -950,10 +950,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.002163944561801226</v>
+        <v>0.002161049652688449</v>
       </c>
       <c r="D18" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="19">
@@ -968,10 +968,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.002266989540934618</v>
+        <v>0.002263956779006946</v>
       </c>
       <c r="D19" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="20">
@@ -986,10 +986,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.002421557009634705</v>
+        <v>0.002418317468484693</v>
       </c>
       <c r="D20" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="21">
@@ -1004,10 +1004,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.002473079499201402</v>
+        <v>0.002469771031643941</v>
       </c>
       <c r="D21" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="22">
@@ -1022,10 +1022,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.002885259415734969</v>
+        <v>0.002881399536917932</v>
       </c>
       <c r="D22" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="23">
@@ -1040,10 +1040,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.002936781905301664</v>
+        <v>0.002932853100077181</v>
       </c>
       <c r="D23" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="24">
@@ -1058,10 +1058,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.004018754186202277</v>
+        <v>0.004013377926421405</v>
       </c>
       <c r="D24" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="25">
@@ -1076,10 +1076,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.004070276675768973</v>
+        <v>0.004064831489580653</v>
       </c>
       <c r="D25" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="26">
@@ -1094,10 +1094,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.004997681487969498</v>
+        <v>0.004990995626447132</v>
       </c>
       <c r="D26" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="27">
@@ -1112,10 +1112,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.005203771446236283</v>
+        <v>0.005196809879084127</v>
       </c>
       <c r="D27" t="n">
-        <v>0.02813127930341594</v>
+        <v>0.02809364548494984</v>
       </c>
     </row>
     <row r="28">
@@ -1130,10 +1130,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.02603279973505632</v>
+        <v>0.02596319156015417</v>
       </c>
       <c r="D28" t="n">
-        <v>0.07809839920516896</v>
+        <v>0.07788957468046249</v>
       </c>
     </row>
     <row r="29">
@@ -1148,10 +1148,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.05538667628419805</v>
+        <v>0.05531258039619243</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1107733525683961</v>
+        <v>0.1106251607923849</v>
       </c>
     </row>
     <row r="30">
@@ -1166,10 +1166,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.1200474006904014</v>
+        <v>0.1198868021610496</v>
       </c>
       <c r="D30" t="n">
-        <v>0.1200474006904014</v>
+        <v>0.1198868021610496</v>
       </c>
     </row>
   </sheetData>
@@ -1183,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1211,523 +1211,145 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>map05217</t>
+          <t>map04979</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Basal cell carcinoma</t>
+          <t>Cholesterol metabolism</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5.152248956669586e-05</v>
+        <v>0.003596748879040124</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00149415219743418</v>
+        <v>0.02877399103232099</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>map04979</t>
+          <t>map04975</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cholesterol metabolism</t>
+          <t>Fat digestion and absorption</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.0005152248956669587</v>
+        <v>0.004673608870762181</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01442629707867484</v>
+        <v>0.03271526209533527</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>map05231</t>
+          <t>map05417</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Choline metabolism in cancer</t>
+          <t>Lipid and atherosclerosis</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0005667473852336546</v>
+        <v>0.005032340450306237</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01530217940130867</v>
+        <v>0.03271526209533527</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>map04927</t>
+          <t>map04148</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cortisol synthesis and secretion</t>
+          <t>Efferocytosis</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.0006182698748003504</v>
+        <v>0.007540359922235842</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01607501674480911</v>
+        <v>0.03770179961117921</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>map04934</t>
+          <t>map04913</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cushing syndrome</t>
+          <t>Ovarian steroidogenesis</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.0006697923643670462</v>
+        <v>0.008613565415143343</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01674480910917615</v>
+        <v>0.03770179961117921</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>map04975</t>
+          <t>map04977</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fat digestion and absorption</t>
+          <t>Vitamin digestion and absorption</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.0006697923643670462</v>
+        <v>0.01503193265827895</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01674480910917615</v>
+        <v>0.04509579797483686</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>map05417</t>
+          <t>map00100</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lipid and atherosclerosis</t>
+          <t>Steroid biosynthesis</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.0007213148539337422</v>
+        <v>0.02035333225062422</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01674480910917615</v>
+        <v>0.04509579797483686</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>map00984</t>
+          <t>map04976</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Steroid degradation</t>
+          <t>Bile secretion</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.0009274048122005254</v>
+        <v>0.03442342291085857</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02040290586841156</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>map04723</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Retrograde endocannabinoid signaling</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0.0009789273017672215</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.02055747333711165</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>map04981</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Folate transport and metabolism</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0.001030449791333917</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.02060899582667835</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>map04148</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Efferocytosis</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>0.001081972280900613</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.02060899582667835</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>map04925</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Aldosterone synthesis and secretion</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>0.001133494770467309</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.02060899582667835</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>map04913</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Ovarian steroidogenesis</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>0.001236539749600701</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.02102117574321191</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>map00981</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Insect hormone biosynthesis</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>0.001288062239167397</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.02102117574321191</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>map00591</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Linoleic acid metabolism</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>0.00149415219743418</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0.0224122829615127</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>map05200</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Pathways in cancer</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>0.001597197176567572</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.0224122829615127</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>map04977</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Vitamin digestion and absorption</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>0.002163944561801226</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>map00592</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>alpha-Linolenic acid metabolism</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>0.002266989540934618</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>map00120</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Primary bile acid biosynthesis</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>0.002421557009634705</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>map01066</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Biosynthesis of alkaloids derived from terpenoid and polyketide</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>0.002473079499201402</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>map00564</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Glycerophospholipid metabolism</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>0.002885259415734969</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>map00100</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Steroid biosynthesis</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>0.002936781905301664</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>map00996</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Biosynthesis of various alkaloids</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>0.004018754186202277</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>map00590</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Arachidonic acid metabolism</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>0.004070276675768973</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>map04976</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Bile secretion</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>0.004997681487969498</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>map00140</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Steroid hormone biosynthesis</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>0.005203771446236283</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0.02813127930341594</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>map01100</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Metabolic pathways</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>0.02603279973505632</v>
-      </c>
-      <c r="D28" t="n">
-        <v>0.07809839920516896</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>map01120</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Microbial metabolism in diverse environments</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>0.05538667628419805</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0.1107733525683961</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>map01110</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Biosynthesis of secondary metabolites</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>0.1200474006904014</v>
-      </c>
-      <c r="D30" t="n">
-        <v>0.1200474006904014</v>
+        <v>0.04509579797483686</v>
       </c>
     </row>
   </sheetData>

</xml_diff>